<commit_message>
Flat DEF with ArmorPen, split herb into Buff table
- UnitStat: ArmorPen column, DEF values rescaled to flat numbers (monsters 0/2/4, boss 4)
- Player: herb columns moved to new Buff table (14001~), common columns first
- Item: statType enum includes ArmorPen, consumable note points to Buff
- README: Formula tab (planner-owned formulas, not exported), Buff, flat DEF rule

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CDH3mwZmVtgx1ALhFj2DHN
</commit_message>
<xml_diff>
--- a/tables/Item.xlsx
+++ b/tables/Item.xlsx
@@ -440,16 +440,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8.380000000000001" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="6.25" customWidth="1" min="3" max="3"/>
     <col width="32.38" customWidth="1" min="6" max="6"/>
-    <col width="6.63" customWidth="1" min="7" max="7"/>
-    <col width="16.75" customWidth="1" min="8" max="8"/>
-    <col width="24.75" customWidth="1" min="9" max="9"/>
+    <col width="7.25" customWidth="1" min="7" max="7"/>
+    <col width="6.63" customWidth="1" min="8" max="8"/>
+    <col width="16.75" customWidth="1" min="9" max="9"/>
     <col width="24.75" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -461,7 +461,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>한 행 = 아이템 하나(무기·방어구·소모품을 한 시트에). ItemType enum: Weapon, Armor, Consumable. StatJson = 그 아이템 스탯 JSON 파일 이름(저장소 stats/item/ 안, 예: 6002.json, 없으면 빈칸). JSON은 [{"statType":"ATK","value":2}] 배열, statType enum = 플레이어 스탯 열 이름과 똑같이(UnitStat의 HP, ATK, DEF, Dodge, Crit, CritMult, Poise, MoveSpeed), value는 정수·비율 만분율. SkillID·AcquireAnim은 무기만. 무기 평타(타수·배율·타이밍)는 데이터로 두지 않고 개발에서 처리, 무기 차이는 StatJson 스탯으로만 줌(10/29). Acquire enum: START, STORY. 상시 사용이라 Active 없음. 무기는 버선칼(시작)·쇠메 2종. 발골칼은 해체 연출용이라 아이템이 아님(6001 비움, 번호 재사용 안 함, 10/29). 방어구·소모품 행과 모든 스탯 값은 예시(10/29, 미확정).</t>
+          <t>한 행 = 아이템 하나(무기·방어구·소모품을 한 시트에). ItemType enum: Weapon, Armor, Consumable. StatJson = 그 아이템 스탯 JSON 파일 이름(저장소 stats/item/ 안, 예: 6002.json, 없으면 빈칸). JSON은 [{"statType":"ATK","value":2}] 배열, statType enum = 플레이어 스탯 열 이름과 똑같이(UnitStat의 HP, ATK, DEF, Dodge, Crit, CritMult, Poise, MoveSpeed, ArmorPen), value는 정수·비율 만분율. 아이템 ATK·ArmorPen은 Formula 탭 데미지 공식에 더해짐. SkillID·AcquireAnim은 무기만. 무기 평타(타수·배율·타이밍)는 데이터로 두지 않고 개발에서 처리, 무기 차이는 StatJson 스탯으로만 줌(10/29). Acquire enum: START, STORY. 상시 사용이라 Active 없음. 무기는 버선칼(시작)·쇠메 2종. 발골칼은 해체 연출용이라 아이템이 아님(6001 비움, 번호 재사용 안 함, 10/29). 방어구·소모품 행과 모든 스탯 값은 예시(10/29, 미확정). 소모품 효과 수치는 Buff 탭.</t>
         </is>
       </c>
       <c r="C1" s="1" t="n"/>
@@ -604,6 +604,7 @@
           <t>Note</t>
         </is>
       </c>
+      <c r="K6" s="2" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="n">
@@ -650,6 +651,7 @@
           <t>시작 무기(10/29 김현호). 스탯 예시: ATK+2, 치명타 확률+2%</t>
         </is>
       </c>
+      <c r="K7" s="3" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="n">
@@ -693,6 +695,7 @@
           <t>완성판. 스탯 예시: ATK+6, 이동 속도-50</t>
         </is>
       </c>
+      <c r="K8" s="3" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n">
@@ -730,6 +733,7 @@
           <t>예시 행. 스탯 예시: 회피+2%, 이동 속도+50</t>
         </is>
       </c>
+      <c r="K9" s="3" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n">
@@ -760,11 +764,13 @@
           <t>STORY</t>
         </is>
       </c>
+      <c r="I10" s="3" t="n"/>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>예시 행. 스탯 예시: HP+40(Player.HerbHeal과 같은 값). 지스타 약초는 Player 탭 값을 씀</t>
-        </is>
-      </c>
+          <t>예시 행. 스탯 예시: HP+40. 실제 회복 수치·사용 횟수는 Buff 14001(10/29)</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n"/>
@@ -773,6 +779,7 @@
       <c r="E11" s="3" t="n"/>
       <c r="F11" s="3" t="n"/>
       <c r="I11" s="3" t="n"/>
+      <c r="K11" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>